<commit_message>
docs: update project design documents
</commit_message>
<xml_diff>
--- a/doc/数据库总表.xlsx
+++ b/doc/数据库总表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080" activeTab="3"/>
+    <workbookView windowWidth="25600" windowHeight="12080" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="DB一览表" sheetId="1" r:id="rId1"/>
@@ -807,7 +807,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -833,17 +833,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="黑体"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1507,19 +1497,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1528,134 +1527,125 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1681,51 +1671,45 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2166,264 +2150,264 @@
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1" spans="1:5">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="18"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16"/>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:5">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:5">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="18" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:5">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="21">
         <v>1</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="22" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:5">
-      <c r="A7" s="25"/>
-      <c r="B7" s="23">
+      <c r="A7" s="23"/>
+      <c r="B7" s="21">
         <v>2</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="22" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:5">
-      <c r="A8" s="25"/>
-      <c r="B8" s="23">
+      <c r="A8" s="23"/>
+      <c r="B8" s="21">
         <v>3</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="22" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:5">
-      <c r="A9" s="25"/>
-      <c r="B9" s="23">
+      <c r="A9" s="23"/>
+      <c r="B9" s="21">
         <v>4</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="22" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:5">
-      <c r="A10" s="25"/>
-      <c r="B10" s="23">
+      <c r="A10" s="23"/>
+      <c r="B10" s="21">
         <v>5</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="22" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:5">
-      <c r="A11" s="25"/>
-      <c r="B11" s="23">
+      <c r="A11" s="23"/>
+      <c r="B11" s="21">
         <v>6</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="22" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:5">
-      <c r="A12" s="25"/>
-      <c r="B12" s="23">
+      <c r="A12" s="23"/>
+      <c r="B12" s="21">
         <v>7</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="22" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:5">
-      <c r="A13" s="25"/>
-      <c r="B13" s="23">
+      <c r="A13" s="23"/>
+      <c r="B13" s="21">
         <v>8</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="22" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:5">
-      <c r="A14" s="25"/>
-      <c r="B14" s="23">
+      <c r="A14" s="23"/>
+      <c r="B14" s="21">
         <v>9</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="22" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1" spans="1:5">
-      <c r="A15" s="25"/>
-      <c r="B15" s="23">
+      <c r="A15" s="23"/>
+      <c r="B15" s="21">
         <v>10</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="24" t="s">
+      <c r="E15" s="22" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:5">
-      <c r="A16" s="25"/>
-      <c r="B16" s="23">
+      <c r="A16" s="23"/>
+      <c r="B16" s="21">
         <v>11</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="D16" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="24" t="s">
+      <c r="E16" s="22" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:5">
-      <c r="A17" s="25"/>
-      <c r="B17" s="23">
+      <c r="A17" s="23"/>
+      <c r="B17" s="21">
         <v>12</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="22" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:5">
-      <c r="A18" s="25"/>
-      <c r="B18" s="23">
+      <c r="A18" s="23"/>
+      <c r="B18" s="21">
         <v>13</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="22" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:5">
-      <c r="A19" s="25"/>
-      <c r="B19" s="23">
+      <c r="A19" s="23"/>
+      <c r="B19" s="21">
         <v>14</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="22" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:5">
-      <c r="A20" s="25"/>
-      <c r="B20" s="23">
+      <c r="A20" s="23"/>
+      <c r="B20" s="21">
         <v>15</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="22" t="s">
         <v>52</v>
       </c>
     </row>
@@ -4513,73 +4497,73 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" spans="1:9">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="13"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="12" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="F4" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="G4" s="15" t="s">
+      <c r="F4" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="H4" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="I4" s="15" t="s">
+      <c r="H4" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="I4" s="13" t="s">
         <v>68</v>
       </c>
     </row>
@@ -4633,13 +4617,13 @@
       <c r="B5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>73</v>
       </c>
       <c r="F5" s="8" t="s">
@@ -4648,13 +4632,13 @@
       <c r="G5" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="8" t="s">
         <v>76</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="8" t="s">
         <v>6</v>
       </c>
     </row>
@@ -4800,7 +4784,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="12" ht="43.5" spans="2:10">
+    <row r="12" ht="14.5" spans="2:10">
       <c r="B12" s="4">
         <v>7</v>
       </c>

</xml_diff>